<commit_message>
Update Refix Debug responder
</commit_message>
<xml_diff>
--- a/data/raw/email_modelos/modelos_resposta_chunks.xlsx
+++ b/data/raw/email_modelos/modelos_resposta_chunks.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P204"/>
+  <dimension ref="A1:P217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14461,10 +14461,10 @@
         <v>1</v>
       </c>
       <c r="K204" s="2" t="n">
-        <v>46262.58553463855</v>
+        <v>46262.58553464121</v>
       </c>
       <c r="L204" s="2" t="n">
-        <v>46262.58553463855</v>
+        <v>46262.58553464121</v>
       </c>
       <c r="M204" t="n">
         <v>2026</v>
@@ -14480,6 +14480,926 @@
           <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
 Assunto tipico: Nota de corte
 Campos a preencher: nome;
+Olá, {{nome}}! Bom dia!
+Nas disciplinas dos cursos de Pós-Graduação EAD da PUC-Campinas, a nota mínima para aprovação é 7,0.
+Caso o aluno obtenha uma nota inferior a 7,0, será considerado reprovado na disciplina e deverá realizar a dependência da matéria para concluir o curso e, posteriormente, emitir o diploma de conclusão.
+Agradecemos a compreensão.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>MOD0185-001</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>MOD0185</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>1</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Alteração de e-mail cadastrado</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Como altero o meu e-mail cadastrado no sistema acadêmico; RES: Alteração de e-mail; Trocar e-mail de contato</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H205" t="b">
+        <v>0</v>
+      </c>
+      <c r="I205" t="n">
+        <v>1</v>
+      </c>
+      <c r="J205" t="n">
+        <v>1</v>
+      </c>
+      <c r="K205" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L205" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M205" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N205" t="n">
+        <v>616</v>
+      </c>
+      <c r="O205" t="n">
+        <v>154</v>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Alteração de e-mail cadastrado
+Campos a preencher: nome
+Olá, {{nome}}!
+Em relação ao seu e-mail pessoal cadastrado, pedimos, por gentileza, que entre em contato diretamente com o PUC Digital pelo e-mail puc-digital@puc-campinas.edu.br para solicitar a alteração.
+Caso a solicitação seja referente ao seu e-mail institucional, informamos que não é possível realizar a alteração, pois esse endereço é gerado automaticamente a partir do seu RA (Registro Acadêmico).
+Agradecemos a compreensão e permanecemos à disposição.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>MOD0186-001</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>MOD0186</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>1</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Envio de atividade no Canvas com prazo expirado</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Como envio uma atividade no Canvas cujo prazo já expirou; Enviar tarefa atrasada no Canvas</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H206" t="b">
+        <v>0</v>
+      </c>
+      <c r="I206" t="n">
+        <v>1</v>
+      </c>
+      <c r="J206" t="n">
+        <v>1</v>
+      </c>
+      <c r="K206" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L206" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M206" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N206" t="n">
+        <v>677</v>
+      </c>
+      <c r="O206" t="n">
+        <v>169</v>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Envio de atividade no Canvas com prazo expirado
+Campos a preencher: nome
+Olá, {{nome}}!
+O Canvas só permite o envio após a data limite quando o professor mantém a atividade aberta para envios atrasados. Se o botão de envio ainda estiver disponível, você pode enviar normalmente e o sistema registrará a entrega como atrasada.
+Caso o envio já esteja bloqueado, entre em contato diretamente com o professor da disciplina para avaliar a reabertura do prazo ou uma forma alternativa de entrega. O puc-digital@puc-campinas dá suporte à plataforma, mas não altera prazos de atividades.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>MOD0187-001</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>MOD0187</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>1</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Envio de tarefas com atraso por motivo médico</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Qual é o procedimento para envio de tarefas com atraso por motivo médico</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H207" t="b">
+        <v>1</v>
+      </c>
+      <c r="I207" t="n">
+        <v>1</v>
+      </c>
+      <c r="J207" t="n">
+        <v>1</v>
+      </c>
+      <c r="K207" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L207" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M207" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N207" t="n">
+        <v>599</v>
+      </c>
+      <c r="O207" t="n">
+        <v>150</v>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Envio de tarefas com atraso por motivo médico
+Campos a preencher: nome
+Olá, {{nome}}!
+A entrega de atividades fora do prazo por motivo de saúde depende da avaliação do professor da disciplina e das normas acadêmicas do seu curso. Orientamos:
+1. Comunicar o professor o quanto antes, anexando o atestado médico.
+2. Protocolar o atestado junto à Secretaria ou Coordenação do seu curso, setor responsável por validar a justificativa e orientar sobre reposição.
+O PUC Digital presta suporte à plataforma 
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>MOD0188-001</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>MOD0188</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>1</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Visualizar a grade curricular do curso</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Como faço para visualizar a grade curricular do meu curso no ambiente virtual; Onde vejo a matriz curricular</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H208" t="b">
+        <v>0</v>
+      </c>
+      <c r="I208" t="n">
+        <v>1</v>
+      </c>
+      <c r="J208" t="n">
+        <v>1</v>
+      </c>
+      <c r="K208" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L208" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M208" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N208" t="n">
+        <v>559</v>
+      </c>
+      <c r="O208" t="n">
+        <v>140</v>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Visualizar a grade curricular do curso
+Campos a preencher: nome
+Olá, {{nome}}!
+A grade curricular (matriz do curso) pode ser consultada no portal acadêmico, na área do aluno, na seção de curso / histórico, e também na página do seu curso no site da PUC-Campinas.
+No Canvas aparecem apenas as disciplinas em que você está matriculado no período atual, e não a matriz completa. Se precisar da matriz oficial para algum trâmite, solicite à Secretaria do seu curso.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>MOD0189-001</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>MOD0189</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>1</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Recuperação de senha e acesso à conta institucional</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Como posso resetar a senha do meu portal acadêmico se esqueci meu e-mail de recuperação; Esqueci minha senha e não consigo entrar no Canvas, como faço para recuperar o acesso; Reset de senha sem e-mail de recuperação</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H209" t="b">
+        <v>1</v>
+      </c>
+      <c r="I209" t="n">
+        <v>1</v>
+      </c>
+      <c r="J209" t="n">
+        <v>1</v>
+      </c>
+      <c r="K209" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L209" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M209" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N209" t="n">
+        <v>610</v>
+      </c>
+      <c r="O209" t="n">
+        <v>152</v>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Recuperação de senha e acesso à conta institucional
+Campos a preencher: nome
+Olá, {{nome}}!
+O acesso ao Canvas e ao portal acadêmico usa a mesma conta institucional da PUC-Campinas. Se você esqueceu a senha e não tem mais acesso ao e-mail de recuperação, a redefinição precisa ser feita pelo PUC Digital:
+- E-mail: puc-digital@puc-campinas.edu.br
+- Informe nome completo, RA e curso para a confirmação de identidade.
+Por segurança da sua conta, não é possível redefinir a senha institucional sem essa validação.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>MOD0190-001</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>MOD0190</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>1</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Consultar notas de semestres anteriores</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Como eu consulto minhas notas do semestre passado</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H210" t="b">
+        <v>0</v>
+      </c>
+      <c r="I210" t="n">
+        <v>1</v>
+      </c>
+      <c r="J210" t="n">
+        <v>1</v>
+      </c>
+      <c r="K210" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L210" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M210" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N210" t="n">
+        <v>557</v>
+      </c>
+      <c r="O210" t="n">
+        <v>139</v>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Consultar notas de semestres anteriores
+Campos a preencher: nome
+Olá, {{nome}}!
+As notas de períodos anteriores ficam no portal acadêmico, na área do aluno, na seção de Disciplina / histórico  / notas e frequência, com filtro por semestre.
+O Canvas mantém apenas as notas lançadas nas disciplinas do período corrente; o registro oficial e histórico é o do portal acadêmico. Se precisar de um histórico com validade oficial, solicite à Secretaria do seu curso.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>MOD0191-001</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>MOD0191</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>1</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Suporte do Canvas para navegador não suportado</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Como funciona o suporte técnico do Canvas para navegador não suportado</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H211" t="b">
+        <v>0</v>
+      </c>
+      <c r="I211" t="n">
+        <v>1</v>
+      </c>
+      <c r="J211" t="n">
+        <v>1</v>
+      </c>
+      <c r="K211" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L211" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M211" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N211" t="n">
+        <v>773</v>
+      </c>
+      <c r="O211" t="n">
+        <v>193</v>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Suporte do Canvas para navegador não suportado
+Campos a preencher: nome
+Olá, {{nome}}!
+O Canvas é compatível com as duas versões mais recentes dos principais navegadores (Google Chrome, Mozilla Firefox, Microsoft Edge e Safari). Se aparecer o aviso de navegador não suportado:
+1. Atualize o navegador para a versão mais recente ou instale um dos navegadores acima.
+2. Limpe o cache e os cookies e faça login novamente.
+3. Teste em uma janela anônima ou em outro dispositivo para isolar o problema.
+Se o aviso persistir mesmo com o navegador atualizado, escreva para puc-digital@puc-campinas.edu.br informando navegador, versão e sistema operacional, com uma captura de tela.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>MOD0192-001</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>MOD0192</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>1</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Pontuação de Atividades Complementares (AACC)</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Como funciona a pontuação por Atividades Complementares (AAC) no meu curso</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H212" t="b">
+        <v>1</v>
+      </c>
+      <c r="I212" t="n">
+        <v>1</v>
+      </c>
+      <c r="J212" t="n">
+        <v>1</v>
+      </c>
+      <c r="K212" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L212" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M212" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N212" t="n">
+        <v>619</v>
+      </c>
+      <c r="O212" t="n">
+        <v>155</v>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Pontuação de Atividades Complementares (AACC)
+Campos a preencher: nome
+Olá, {{nome}}!
+As regras de Atividades Acadêmico-Científico-Culturais (AACC) — carga horária total exigida, categorias aceitas, limites por tipo de atividade e forma de comprovação — são definidas pelo Projeto Pedagógico de cada curso.
+Para o seu caso, consulte o regulamento de AACC do seu curso (disponível com a Coordenação) e faça o registro e a validação das horas junto à Secretaria ou Coordenação. O PUC Digital não faz o cômputo dessas horas.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>MOD0193-001</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>MOD0193</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>1</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Trancamento de disciplina ou do curso</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Posso trancar uma disciplina?; É possível trancar o curso?; Quero trancar minha pós-graduação; Como faço para trancar uma matéria?</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H213" t="b">
+        <v>1</v>
+      </c>
+      <c r="I213" t="n">
+        <v>1</v>
+      </c>
+      <c r="J213" t="n">
+        <v>1</v>
+      </c>
+      <c r="K213" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L213" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M213" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N213" t="n">
+        <v>886</v>
+      </c>
+      <c r="O213" t="n">
+        <v>222</v>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Trancamento de disciplina ou do curso
+Campos a preencher: nome
+Olá, {{nome}}!
+Informamos que não é possível realizar o trancamento individual de uma disciplina nem o trancamento do curso.
+Caso o aluno não possa continuar os estudos, é possível solicitar o cancelamento do curso. Posteriormente, caso queira retornar, poderá realizar uma nova matrícula no curso e solicitar o aproveitamento das disciplinas que já foram concluídas e aprovadas, conforme as regras da instituição.
+Dessa forma, as disciplinas já realizadas e aprovadas poderão ser consideradas no retorno, não sendo necessário cursá-las novamente, desde que atendam aos critérios de aproveitamento.
+Em caso de dúvidas sobre o cancelamento ou uma futura rematrícula, recomendamos entrar em contato com a Secretaria do curso.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>MOD0194-001</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>MOD0194</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>1</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Reagendamento de prova substitutiva</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Como faço para reagendar uma prova substitutiva que perdi</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H214" t="b">
+        <v>1</v>
+      </c>
+      <c r="I214" t="n">
+        <v>1</v>
+      </c>
+      <c r="J214" t="n">
+        <v>1</v>
+      </c>
+      <c r="K214" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L214" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M214" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N214" t="n">
+        <v>549</v>
+      </c>
+      <c r="O214" t="n">
+        <v>137</v>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Reagendamento de prova substitutiva
+Campos a preencher: nome
+Olá, {{nome}}!
+A solicitação e o agendamento de prova substitutiva (segunda chamada) são feitos junto ao professor da disciplina e à Secretaria ou Coordenação do seu curso, dentro do prazo previsto no regulamento, geralmente mediante justificativa e documento comprobatório.
+O PUC Digital dá suporte à plataforma, mas não agenda avaliações. Procure a Secretaria do seu curso o quanto antes.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>MOD0195-001</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>MOD0195</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>1</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Matrícula em disciplina isolada</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Como faço a matrícula de uma depedencia; Solicito DP</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H215" t="b">
+        <v>1</v>
+      </c>
+      <c r="I215" t="n">
+        <v>1</v>
+      </c>
+      <c r="J215" t="n">
+        <v>1</v>
+      </c>
+      <c r="K215" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L215" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M215" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N215" t="n">
+        <v>502</v>
+      </c>
+      <c r="O215" t="n">
+        <v>126</v>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Matrícula em disciplina isolada
+Campos a preencher: nome
+Olá, {{nome}}!
+A matrícula em disciplina  — cursos que a oferecem, período de solicitação, número de vagas e valores — é tratada pela Secretaria Acadêmica e pela coordenação do curso responsável pela disciplina.
+Entre em contato com puc-digital@puc-campinas.edu.br de interesse para verificar a disponibilidade e o procedimento no período vigente.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>MOD0196-001</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>MOD0196</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>1</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Datas do calendário acadêmico</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Quais são as datas exatas do calendário acadêmico deste semestre</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H216" t="b">
+        <v>1</v>
+      </c>
+      <c r="I216" t="n">
+        <v>1</v>
+      </c>
+      <c r="J216" t="n">
+        <v>1</v>
+      </c>
+      <c r="K216" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L216" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M216" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N216" t="n">
+        <v>360</v>
+      </c>
+      <c r="O216" t="n">
+        <v>90</v>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Datas do calendário acadêmico
+Campos a preencher: nome
+Olá, {{nome}}!
+As datas oficiais do calendário acadêmico são publicadas no site da PUC-Campinas nesse link:https://www.puc-campinas.edu.br/calendario/. A Puc-digital também pode informar as datas específicas.
+Atenciosamente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>MOD0197-001</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>MOD0197</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>1</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Nota de corte</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Nota de aprovação; nota minima para aprovacao</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H217" t="b">
+        <v>0</v>
+      </c>
+      <c r="I217" t="n">
+        <v>1</v>
+      </c>
+      <c r="J217" t="n">
+        <v>1</v>
+      </c>
+      <c r="K217" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="L217" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="M217" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N217" t="n">
+        <v>491</v>
+      </c>
+      <c r="O217" t="n">
+        <v>123</v>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>Modelo de resposta padrao do suporte (usado 1x em 1 thread).
+Assunto tipico: Nota de corte
+Campos a preencher: nome
 Olá, {{nome}}! Bom dia!
 Nas disciplinas dos cursos de Pós-Graduação EAD da PUC-Campinas, a nota mínima para aprovação é 7,0.
 Caso o aluno obtenha uma nota inferior a 7,0, será considerado reprovado na disciplina e deverá realizar a dependência da matéria para concluir o curso e, posteriormente, emitir o diploma de conclusão.
@@ -14499,7 +15419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K185"/>
+  <dimension ref="A1:K198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23627,10 +24547,10 @@
         <v>1</v>
       </c>
       <c r="E185" s="2" t="n">
-        <v>46262.58553463855</v>
+        <v>46262.58553464121</v>
       </c>
       <c r="F185" s="2" t="n">
-        <v>46262.58553463855</v>
+        <v>46262.58553464121</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -23656,6 +24576,614 @@
         <v>0</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>MOD0185</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Alteração de e-mail cadastrado</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>1</v>
+      </c>
+      <c r="D186" t="n">
+        <v>1</v>
+      </c>
+      <c r="E186" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F186" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Como altero o meu e-mail cadastrado no sistema acadêmico; RES: Alteração de e-mail; Trocar e-mail de contato</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+Em relação ao seu e-mail pessoal cadastrado, pedimos, por gentileza, que entre em contato diretamente com o PUC Digital pelo e-mail puc-digital@puc-campinas.edu.br para solicitar a alteração.
+Caso a solicitação seja referente ao seu e-mail institucional, informamos que não é possível realizar a alteração, pois esse endereço é gerado automaticamente a partir do seu RA (Registro Acadêmico).
+Agradecemos a compreensão e permanecemos à disposição.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K186" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>MOD0186</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Envio de atividade no Canvas com prazo expirado</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>1</v>
+      </c>
+      <c r="D187" t="n">
+        <v>1</v>
+      </c>
+      <c r="E187" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F187" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Como envio uma atividade no Canvas cujo prazo já expirou; Enviar tarefa atrasada no Canvas</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr"/>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+O Canvas só permite o envio após a data limite quando o professor mantém a atividade aberta para envios atrasados. Se o botão de envio ainda estiver disponível, você pode enviar normalmente e o sistema registrará a entrega como atrasada.
+Caso o envio já esteja bloqueado, entre em contato diretamente com o professor da disciplina para avaliar a reabertura do prazo ou uma forma alternativa de entrega. O puc-digital@puc-campinas dá suporte à plataforma, mas não altera prazos de atividades.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K187" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>MOD0187</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Envio de tarefas com atraso por motivo médico</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>1</v>
+      </c>
+      <c r="D188" t="n">
+        <v>1</v>
+      </c>
+      <c r="E188" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F188" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Qual é o procedimento para envio de tarefas com atraso por motivo médico</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+A entrega de atividades fora do prazo por motivo de saúde depende da avaliação do professor da disciplina e das normas acadêmicas do seu curso. Orientamos:
+1. Comunicar o professor o quanto antes, anexando o atestado médico.
+2. Protocolar o atestado junto à Secretaria ou Coordenação do seu curso, setor responsável por validar a justificativa e orientar sobre reposição.
+O PUC Digital presta suporte à plataforma 
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K188" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>MOD0188</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Visualizar a grade curricular do curso</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>1</v>
+      </c>
+      <c r="D189" t="n">
+        <v>1</v>
+      </c>
+      <c r="E189" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F189" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Como faço para visualizar a grade curricular do meu curso no ambiente virtual; Onde vejo a matriz curricular</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr"/>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+A grade curricular (matriz do curso) pode ser consultada no portal acadêmico, na área do aluno, na seção de curso / histórico, e também na página do seu curso no site da PUC-Campinas.
+No Canvas aparecem apenas as disciplinas em que você está matriculado no período atual, e não a matriz completa. Se precisar da matriz oficial para algum trâmite, solicite à Secretaria do seu curso.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K189" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>MOD0189</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Recuperação de senha e acesso à conta institucional</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>1</v>
+      </c>
+      <c r="D190" t="n">
+        <v>1</v>
+      </c>
+      <c r="E190" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F190" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Como posso resetar a senha do meu portal acadêmico se esqueci meu e-mail de recuperação; Esqueci minha senha e não consigo entrar no Canvas, como faço para recuperar o acesso; Reset de senha sem e-mail de recuperação</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr"/>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+O acesso ao Canvas e ao portal acadêmico usa a mesma conta institucional da PUC-Campinas. Se você esqueceu a senha e não tem mais acesso ao e-mail de recuperação, a redefinição precisa ser feita pelo PUC Digital:
+- E-mail: puc-digital@puc-campinas.edu.br
+- Informe nome completo, RA e curso para a confirmação de identidade.
+Por segurança da sua conta, não é possível redefinir a senha institucional sem essa validação.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K190" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>MOD0190</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Consultar notas de semestres anteriores</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>1</v>
+      </c>
+      <c r="D191" t="n">
+        <v>1</v>
+      </c>
+      <c r="E191" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F191" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Como eu consulto minhas notas do semestre passado</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+As notas de períodos anteriores ficam no portal acadêmico, na área do aluno, na seção de Disciplina / histórico  / notas e frequência, com filtro por semestre.
+O Canvas mantém apenas as notas lançadas nas disciplinas do período corrente; o registro oficial e histórico é o do portal acadêmico. Se precisar de um histórico com validade oficial, solicite à Secretaria do seu curso.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K191" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>MOD0191</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Suporte do Canvas para navegador não suportado</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>1</v>
+      </c>
+      <c r="D192" t="n">
+        <v>1</v>
+      </c>
+      <c r="E192" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F192" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Como funciona o suporte técnico do Canvas para navegador não suportado</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr"/>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+O Canvas é compatível com as duas versões mais recentes dos principais navegadores (Google Chrome, Mozilla Firefox, Microsoft Edge e Safari). Se aparecer o aviso de navegador não suportado:
+1. Atualize o navegador para a versão mais recente ou instale um dos navegadores acima.
+2. Limpe o cache e os cookies e faça login novamente.
+3. Teste em uma janela anônima ou em outro dispositivo para isolar o problema.
+Se o aviso persistir mesmo com o navegador atualizado, escreva para puc-digital@puc-campinas.edu.br informando navegador, versão e sistema operacional, com uma captura de tela.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K192" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>MOD0192</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Pontuação de Atividades Complementares (AACC)</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>1</v>
+      </c>
+      <c r="D193" t="n">
+        <v>1</v>
+      </c>
+      <c r="E193" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F193" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Como funciona a pontuação por Atividades Complementares (AAC) no meu curso</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr"/>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+As regras de Atividades Acadêmico-Científico-Culturais (AACC) — carga horária total exigida, categorias aceitas, limites por tipo de atividade e forma de comprovação — são definidas pelo Projeto Pedagógico de cada curso.
+Para o seu caso, consulte o regulamento de AACC do seu curso (disponível com a Coordenação) e faça o registro e a validação das horas junto à Secretaria ou Coordenação. O PUC Digital não faz o cômputo dessas horas.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K193" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>MOD0193</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Trancamento de disciplina ou do curso</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>1</v>
+      </c>
+      <c r="D194" t="n">
+        <v>1</v>
+      </c>
+      <c r="E194" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F194" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Posso trancar uma disciplina?; É possível trancar o curso?; Quero trancar minha pós-graduação; Como faço para trancar uma matéria?</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+Informamos que não é possível realizar o trancamento individual de uma disciplina nem o trancamento do curso.
+Caso o aluno não possa continuar os estudos, é possível solicitar o cancelamento do curso. Posteriormente, caso queira retornar, poderá realizar uma nova matrícula no curso e solicitar o aproveitamento das disciplinas que já foram concluídas e aprovadas, conforme as regras da instituição.
+Dessa forma, as disciplinas já realizadas e aprovadas poderão ser consideradas no retorno, não sendo necessário cursá-las novamente, desde que atendam aos critérios de aproveitamento.
+Em caso de dúvidas sobre o cancelamento ou uma futura rematrícula, recomendamos entrar em contato com a Secretaria do curso.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K194" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>MOD0194</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Reagendamento de prova substitutiva</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>1</v>
+      </c>
+      <c r="D195" t="n">
+        <v>1</v>
+      </c>
+      <c r="E195" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F195" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Como faço para reagendar uma prova substitutiva que perdi</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr"/>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+A solicitação e o agendamento de prova substitutiva (segunda chamada) são feitos junto ao professor da disciplina e à Secretaria ou Coordenação do seu curso, dentro do prazo previsto no regulamento, geralmente mediante justificativa e documento comprobatório.
+O PUC Digital dá suporte à plataforma, mas não agenda avaliações. Procure a Secretaria do seu curso o quanto antes.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K195" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>MOD0195</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Matrícula em disciplina isolada</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>1</v>
+      </c>
+      <c r="D196" t="n">
+        <v>1</v>
+      </c>
+      <c r="E196" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F196" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Como faço a matrícula de uma depedencia; Solicito DP</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr"/>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+A matrícula em disciplina  — cursos que a oferecem, período de solicitação, número de vagas e valores — é tratada pela Secretaria Acadêmica e pela coordenação do curso responsável pela disciplina.
+Entre em contato com puc-digital@puc-campinas.edu.br de interesse para verificar a disponibilidade e o procedimento no período vigente.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K196" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>MOD0196</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Datas do calendário acadêmico</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>1</v>
+      </c>
+      <c r="D197" t="n">
+        <v>1</v>
+      </c>
+      <c r="E197" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F197" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Quais são as datas exatas do calendário acadêmico deste semestre</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr"/>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}!
+As datas oficiais do calendário acadêmico são publicadas no site da PUC-Campinas nesse link:https://www.puc-campinas.edu.br/calendario/. A Puc-digital também pode informar as datas específicas.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K197" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>MOD0197</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Nota de corte</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>1</v>
+      </c>
+      <c r="D198" t="n">
+        <v>1</v>
+      </c>
+      <c r="E198" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="F198" s="2" t="n">
+        <v>46275.56229148144</v>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Nota de aprovação; nota minima para aprovacao</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr"/>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Olá, {{nome}}! Bom dia!
+Nas disciplinas dos cursos de Pós-Graduação EAD da PUC-Campinas, a nota mínima para aprovação é 7,0.
+Caso o aluno obtenha uma nota inferior a 7,0, será considerado reprovado na disciplina e deverá realizar a dependência da matéria para concluir o curso e, posteriormente, emitir o diploma de conclusão.
+Agradecemos a compreensão.
+Atenciosamente,</t>
+        </is>
+      </c>
+      <c r="K198" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>